<commit_message>
fix: remove practice exam from courseware
</commit_message>
<xml_diff>
--- a/activities/activity-05-measure-project-profitability-and-billing-leakage/activity-05-control.xlsx
+++ b/activities/activity-05-measure-project-profitability-and-billing-leakage/activity-05-control.xlsx
@@ -712,11 +712,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="15982753"/>
-        <c:axId val="82217544"/>
+        <c:axId val="95134788"/>
+        <c:axId val="40013464"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="15982753"/>
+        <c:axId val="95134788"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -749,7 +749,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82217544"/>
+        <c:crossAx val="40013464"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -757,7 +757,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82217544"/>
+        <c:axId val="40013464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -833,7 +833,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15982753"/>
+        <c:crossAx val="95134788"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>